<commit_message>
fix: layout identico al foglio di riferimento, test di confronto, interfaccia in italiano
</commit_message>
<xml_diff>
--- a/esempi/movimenti_GBP_eur.xlsx
+++ b/esempi/movimenti_GBP_eur.xlsx
@@ -54,10 +54,11 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="3">
+  <cellXfs count="4">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="165" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="1" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -423,7 +424,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L47"/>
+  <dimension ref="A1:P47"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="18" customWidth="1" min="1" max="1"/>
@@ -438,6 +439,10 @@
     <col width="18" customWidth="1" min="10" max="10"/>
     <col width="18" customWidth="1" min="11" max="11"/>
     <col width="18" customWidth="1" min="12" max="12"/>
+    <col width="18" customWidth="1" min="13" max="13"/>
+    <col width="18" customWidth="1" min="14" max="14"/>
+    <col width="18" customWidth="1" min="15" max="15"/>
+    <col width="18" customWidth="1" min="16" max="16"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -453,52 +458,64 @@
       </c>
       <c r="C1" s="1" t="inlineStr">
         <is>
-          <t>entrate (GBP)</t>
+          <t>entrate</t>
         </is>
       </c>
       <c r="D1" s="1" t="inlineStr">
         <is>
-          <t>uscite (GBP)</t>
+          <t>uscite</t>
         </is>
       </c>
       <c r="E1" s="1" t="inlineStr">
         <is>
-          <t>saldo (GBP)</t>
+          <t>saldo</t>
         </is>
       </c>
       <c r="F1" s="1" t="inlineStr">
         <is>
+          <t>gg</t>
+        </is>
+      </c>
+      <c r="G1" s="1" t="inlineStr">
+        <is>
+          <t>saldo x gg</t>
+        </is>
+      </c>
+      <c r="H1" s="1" t="n"/>
+      <c r="I1" s="1" t="inlineStr">
+        <is>
           <t>cambio</t>
         </is>
       </c>
-      <c r="G1" s="1" t="inlineStr">
+      <c r="J1" s="1" t="inlineStr">
+        <is>
+          <t>entrate in euro</t>
+        </is>
+      </c>
+      <c r="K1" s="1" t="inlineStr">
+        <is>
+          <t>uscite in euro</t>
+        </is>
+      </c>
+      <c r="L1" s="1" t="inlineStr">
+        <is>
+          <t>saldo in euro</t>
+        </is>
+      </c>
+      <c r="M1" s="1" t="inlineStr">
+        <is>
+          <t>gg</t>
+        </is>
+      </c>
+      <c r="N1" s="1" t="inlineStr">
+        <is>
+          <t>saldo x gg in euro</t>
+        </is>
+      </c>
+      <c r="O1" s="1" t="n"/>
+      <c r="P1" s="1" t="inlineStr">
         <is>
           <t>data cambio usata</t>
-        </is>
-      </c>
-      <c r="H1" s="1" t="inlineStr">
-        <is>
-          <t>entrate (EUR)</t>
-        </is>
-      </c>
-      <c r="I1" s="1" t="inlineStr">
-        <is>
-          <t>uscite (EUR)</t>
-        </is>
-      </c>
-      <c r="J1" s="1" t="inlineStr">
-        <is>
-          <t>saldo (EUR)</t>
-        </is>
-      </c>
-      <c r="K1" s="1" t="inlineStr">
-        <is>
-          <t>gg</t>
-        </is>
-      </c>
-      <c r="L1" s="1" t="inlineStr">
-        <is>
-          <t>saldo x gg (EUR)</t>
         </is>
       </c>
     </row>
@@ -515,37 +532,41 @@
         <v>1605.36</v>
       </c>
       <c r="E2">
-        <f>N(C2)-N(D2)</f>
-        <v/>
-      </c>
-      <c r="F2">
+        <f>C2-D2</f>
+        <v/>
+      </c>
+      <c r="F2" s="3">
+        <f>DAYS(A3,A2)</f>
+        <v/>
+      </c>
+      <c r="G2">
+        <f>F2*E2</f>
+        <v/>
+      </c>
+      <c r="I2">
         <f>'Medie mensili'!C2</f>
         <v/>
       </c>
-      <c r="G2" s="2" t="inlineStr">
+      <c r="J2">
+        <f>C2/I2</f>
+        <v/>
+      </c>
+      <c r="L2">
+        <f>J2-K2</f>
+        <v/>
+      </c>
+      <c r="M2" s="3">
+        <f>F2</f>
+        <v/>
+      </c>
+      <c r="N2">
+        <f>M2*L2</f>
+        <v/>
+      </c>
+      <c r="P2" s="2" t="inlineStr">
         <is>
           <t>media mensile</t>
         </is>
-      </c>
-      <c r="H2">
-        <f>IF(C2="","",C2/F2)</f>
-        <v/>
-      </c>
-      <c r="I2">
-        <f>IF(D2="","",D2/F2)</f>
-        <v/>
-      </c>
-      <c r="J2">
-        <f>N(H2)-N(I2)</f>
-        <v/>
-      </c>
-      <c r="K2">
-        <f>A3-A2</f>
-        <v/>
-      </c>
-      <c r="L2">
-        <f>K2*J2</f>
-        <v/>
       </c>
     </row>
     <row r="3">
@@ -557,35 +578,39 @@
         <v>1000</v>
       </c>
       <c r="E3">
-        <f>E2+N(C3)-N(D3)</f>
-        <v/>
-      </c>
-      <c r="F3">
+        <f>E2+C3-D3</f>
+        <v/>
+      </c>
+      <c r="F3" s="3">
+        <f>DAYS(A4,A3)</f>
+        <v/>
+      </c>
+      <c r="G3">
+        <f>F3*E3</f>
+        <v/>
+      </c>
+      <c r="I3">
         <f>LOOKUP(A3,Cambi!$A$2:$A$255,Cambi!$B$2:$B$255)</f>
         <v/>
       </c>
-      <c r="G3" s="2">
+      <c r="J3">
+        <f>C3/I3</f>
+        <v/>
+      </c>
+      <c r="L3">
+        <f>L2+J3-K3</f>
+        <v/>
+      </c>
+      <c r="M3" s="3">
+        <f>F3</f>
+        <v/>
+      </c>
+      <c r="N3">
+        <f>M3*L3</f>
+        <v/>
+      </c>
+      <c r="P3" s="2">
         <f>LOOKUP(A3,Cambi!$A$2:$A$255,Cambi!$A$2:$A$255)</f>
-        <v/>
-      </c>
-      <c r="H3">
-        <f>IF(C3="","",C3/F3)</f>
-        <v/>
-      </c>
-      <c r="I3">
-        <f>IF(D3="","",D3/F3)</f>
-        <v/>
-      </c>
-      <c r="J3">
-        <f>J2+N(H3)-N(I3)</f>
-        <v/>
-      </c>
-      <c r="K3">
-        <f>A4-A3</f>
-        <v/>
-      </c>
-      <c r="L3">
-        <f>K3*J3</f>
         <v/>
       </c>
     </row>
@@ -598,35 +623,39 @@
         <v>2500</v>
       </c>
       <c r="E4">
-        <f>E3+N(C4)-N(D4)</f>
-        <v/>
-      </c>
-      <c r="F4">
+        <f>E3+C4-D4</f>
+        <v/>
+      </c>
+      <c r="F4" s="3">
+        <f>DAYS(A5,A4)</f>
+        <v/>
+      </c>
+      <c r="G4">
+        <f>F4*E4</f>
+        <v/>
+      </c>
+      <c r="I4">
         <f>LOOKUP(A4,Cambi!$A$2:$A$255,Cambi!$B$2:$B$255)</f>
         <v/>
       </c>
-      <c r="G4" s="2">
+      <c r="J4">
+        <f>C4/I4</f>
+        <v/>
+      </c>
+      <c r="L4">
+        <f>L3+J4-K4</f>
+        <v/>
+      </c>
+      <c r="M4" s="3">
+        <f>F4</f>
+        <v/>
+      </c>
+      <c r="N4">
+        <f>M4*L4</f>
+        <v/>
+      </c>
+      <c r="P4" s="2">
         <f>LOOKUP(A4,Cambi!$A$2:$A$255,Cambi!$A$2:$A$255)</f>
-        <v/>
-      </c>
-      <c r="H4">
-        <f>IF(C4="","",C4/F4)</f>
-        <v/>
-      </c>
-      <c r="I4">
-        <f>IF(D4="","",D4/F4)</f>
-        <v/>
-      </c>
-      <c r="J4">
-        <f>J3+N(H4)-N(I4)</f>
-        <v/>
-      </c>
-      <c r="K4">
-        <f>A5-A4</f>
-        <v/>
-      </c>
-      <c r="L4">
-        <f>K4*J4</f>
         <v/>
       </c>
     </row>
@@ -639,35 +668,39 @@
         <v>3000</v>
       </c>
       <c r="E5">
-        <f>E4+N(C5)-N(D5)</f>
-        <v/>
-      </c>
-      <c r="F5">
+        <f>E4+C5-D5</f>
+        <v/>
+      </c>
+      <c r="F5" s="3">
+        <f>DAYS(A6,A5)</f>
+        <v/>
+      </c>
+      <c r="G5">
+        <f>F5*E5</f>
+        <v/>
+      </c>
+      <c r="I5">
         <f>LOOKUP(A5,Cambi!$A$2:$A$255,Cambi!$B$2:$B$255)</f>
         <v/>
       </c>
-      <c r="G5" s="2">
+      <c r="K5">
+        <f>D5/I5</f>
+        <v/>
+      </c>
+      <c r="L5">
+        <f>L4+J5-K5</f>
+        <v/>
+      </c>
+      <c r="M5" s="3">
+        <f>F5</f>
+        <v/>
+      </c>
+      <c r="N5">
+        <f>M5*L5</f>
+        <v/>
+      </c>
+      <c r="P5" s="2">
         <f>LOOKUP(A5,Cambi!$A$2:$A$255,Cambi!$A$2:$A$255)</f>
-        <v/>
-      </c>
-      <c r="H5">
-        <f>IF(C5="","",C5/F5)</f>
-        <v/>
-      </c>
-      <c r="I5">
-        <f>IF(D5="","",D5/F5)</f>
-        <v/>
-      </c>
-      <c r="J5">
-        <f>J4+N(H5)-N(I5)</f>
-        <v/>
-      </c>
-      <c r="K5">
-        <f>A6-A5</f>
-        <v/>
-      </c>
-      <c r="L5">
-        <f>K5*J5</f>
         <v/>
       </c>
     </row>
@@ -680,35 +713,39 @@
         <v>600</v>
       </c>
       <c r="E6">
-        <f>E5+N(C6)-N(D6)</f>
-        <v/>
-      </c>
-      <c r="F6">
+        <f>E5+C6-D6</f>
+        <v/>
+      </c>
+      <c r="F6" s="3">
+        <f>DAYS(A7,A6)</f>
+        <v/>
+      </c>
+      <c r="G6">
+        <f>F6*E6</f>
+        <v/>
+      </c>
+      <c r="I6">
         <f>LOOKUP(A6,Cambi!$A$2:$A$255,Cambi!$B$2:$B$255)</f>
         <v/>
       </c>
-      <c r="G6" s="2">
+      <c r="J6">
+        <f>C6/I6</f>
+        <v/>
+      </c>
+      <c r="L6">
+        <f>L5+J6-K6</f>
+        <v/>
+      </c>
+      <c r="M6" s="3">
+        <f>F6</f>
+        <v/>
+      </c>
+      <c r="N6">
+        <f>M6*L6</f>
+        <v/>
+      </c>
+      <c r="P6" s="2">
         <f>LOOKUP(A6,Cambi!$A$2:$A$255,Cambi!$A$2:$A$255)</f>
-        <v/>
-      </c>
-      <c r="H6">
-        <f>IF(C6="","",C6/F6)</f>
-        <v/>
-      </c>
-      <c r="I6">
-        <f>IF(D6="","",D6/F6)</f>
-        <v/>
-      </c>
-      <c r="J6">
-        <f>J5+N(H6)-N(I6)</f>
-        <v/>
-      </c>
-      <c r="K6">
-        <f>A7-A6</f>
-        <v/>
-      </c>
-      <c r="L6">
-        <f>K6*J6</f>
         <v/>
       </c>
     </row>
@@ -721,35 +758,39 @@
         <v>14824.2</v>
       </c>
       <c r="E7">
-        <f>E6+N(C7)-N(D7)</f>
-        <v/>
-      </c>
-      <c r="F7">
+        <f>E6+C7-D7</f>
+        <v/>
+      </c>
+      <c r="F7" s="3">
+        <f>DAYS(A8,A7)</f>
+        <v/>
+      </c>
+      <c r="G7">
+        <f>F7*E7</f>
+        <v/>
+      </c>
+      <c r="I7">
         <f>LOOKUP(A7,Cambi!$A$2:$A$255,Cambi!$B$2:$B$255)</f>
         <v/>
       </c>
-      <c r="G7" s="2">
+      <c r="J7">
+        <f>C7/I7</f>
+        <v/>
+      </c>
+      <c r="L7">
+        <f>L6+J7-K7</f>
+        <v/>
+      </c>
+      <c r="M7" s="3">
+        <f>F7</f>
+        <v/>
+      </c>
+      <c r="N7">
+        <f>M7*L7</f>
+        <v/>
+      </c>
+      <c r="P7" s="2">
         <f>LOOKUP(A7,Cambi!$A$2:$A$255,Cambi!$A$2:$A$255)</f>
-        <v/>
-      </c>
-      <c r="H7">
-        <f>IF(C7="","",C7/F7)</f>
-        <v/>
-      </c>
-      <c r="I7">
-        <f>IF(D7="","",D7/F7)</f>
-        <v/>
-      </c>
-      <c r="J7">
-        <f>J6+N(H7)-N(I7)</f>
-        <v/>
-      </c>
-      <c r="K7">
-        <f>A8-A7</f>
-        <v/>
-      </c>
-      <c r="L7">
-        <f>K7*J7</f>
         <v/>
       </c>
     </row>
@@ -762,35 +803,39 @@
         <v>14824.2</v>
       </c>
       <c r="E8">
-        <f>E7+N(C8)-N(D8)</f>
-        <v/>
-      </c>
-      <c r="F8">
+        <f>E7+C8-D8</f>
+        <v/>
+      </c>
+      <c r="F8" s="3">
+        <f>DAYS(A9,A8)</f>
+        <v/>
+      </c>
+      <c r="G8">
+        <f>F8*E8</f>
+        <v/>
+      </c>
+      <c r="I8">
         <f>LOOKUP(A8,Cambi!$A$2:$A$255,Cambi!$B$2:$B$255)</f>
         <v/>
       </c>
-      <c r="G8" s="2">
+      <c r="K8">
+        <f>D8/I8</f>
+        <v/>
+      </c>
+      <c r="L8">
+        <f>L7+J8-K8</f>
+        <v/>
+      </c>
+      <c r="M8" s="3">
+        <f>F8</f>
+        <v/>
+      </c>
+      <c r="N8">
+        <f>M8*L8</f>
+        <v/>
+      </c>
+      <c r="P8" s="2">
         <f>LOOKUP(A8,Cambi!$A$2:$A$255,Cambi!$A$2:$A$255)</f>
-        <v/>
-      </c>
-      <c r="H8">
-        <f>IF(C8="","",C8/F8)</f>
-        <v/>
-      </c>
-      <c r="I8">
-        <f>IF(D8="","",D8/F8)</f>
-        <v/>
-      </c>
-      <c r="J8">
-        <f>J7+N(H8)-N(I8)</f>
-        <v/>
-      </c>
-      <c r="K8">
-        <f>A9-A8</f>
-        <v/>
-      </c>
-      <c r="L8">
-        <f>K8*J8</f>
         <v/>
       </c>
     </row>
@@ -803,35 +848,39 @@
         <v>1276</v>
       </c>
       <c r="E9">
-        <f>E8+N(C9)-N(D9)</f>
-        <v/>
-      </c>
-      <c r="F9">
+        <f>E8+C9-D9</f>
+        <v/>
+      </c>
+      <c r="F9" s="3">
+        <f>DAYS(A10,A9)</f>
+        <v/>
+      </c>
+      <c r="G9">
+        <f>F9*E9</f>
+        <v/>
+      </c>
+      <c r="I9">
         <f>LOOKUP(A9,Cambi!$A$2:$A$255,Cambi!$B$2:$B$255)</f>
         <v/>
       </c>
-      <c r="G9" s="2">
+      <c r="K9">
+        <f>D9/I9</f>
+        <v/>
+      </c>
+      <c r="L9">
+        <f>L8+J9-K9</f>
+        <v/>
+      </c>
+      <c r="M9" s="3">
+        <f>F9</f>
+        <v/>
+      </c>
+      <c r="N9">
+        <f>M9*L9</f>
+        <v/>
+      </c>
+      <c r="P9" s="2">
         <f>LOOKUP(A9,Cambi!$A$2:$A$255,Cambi!$A$2:$A$255)</f>
-        <v/>
-      </c>
-      <c r="H9">
-        <f>IF(C9="","",C9/F9)</f>
-        <v/>
-      </c>
-      <c r="I9">
-        <f>IF(D9="","",D9/F9)</f>
-        <v/>
-      </c>
-      <c r="J9">
-        <f>J8+N(H9)-N(I9)</f>
-        <v/>
-      </c>
-      <c r="K9">
-        <f>A10-A9</f>
-        <v/>
-      </c>
-      <c r="L9">
-        <f>K9*J9</f>
         <v/>
       </c>
     </row>
@@ -844,35 +893,39 @@
         <v>1000</v>
       </c>
       <c r="E10">
-        <f>E9+N(C10)-N(D10)</f>
-        <v/>
-      </c>
-      <c r="F10">
+        <f>E9+C10-D10</f>
+        <v/>
+      </c>
+      <c r="F10" s="3">
+        <f>DAYS(A11,A10)</f>
+        <v/>
+      </c>
+      <c r="G10">
+        <f>F10*E10</f>
+        <v/>
+      </c>
+      <c r="I10">
         <f>LOOKUP(A10,Cambi!$A$2:$A$255,Cambi!$B$2:$B$255)</f>
         <v/>
       </c>
-      <c r="G10" s="2">
+      <c r="J10">
+        <f>C10/I10</f>
+        <v/>
+      </c>
+      <c r="L10">
+        <f>L9+J10-K10</f>
+        <v/>
+      </c>
+      <c r="M10" s="3">
+        <f>F10</f>
+        <v/>
+      </c>
+      <c r="N10">
+        <f>M10*L10</f>
+        <v/>
+      </c>
+      <c r="P10" s="2">
         <f>LOOKUP(A10,Cambi!$A$2:$A$255,Cambi!$A$2:$A$255)</f>
-        <v/>
-      </c>
-      <c r="H10">
-        <f>IF(C10="","",C10/F10)</f>
-        <v/>
-      </c>
-      <c r="I10">
-        <f>IF(D10="","",D10/F10)</f>
-        <v/>
-      </c>
-      <c r="J10">
-        <f>J9+N(H10)-N(I10)</f>
-        <v/>
-      </c>
-      <c r="K10">
-        <f>A11-A10</f>
-        <v/>
-      </c>
-      <c r="L10">
-        <f>K10*J10</f>
         <v/>
       </c>
     </row>
@@ -885,35 +938,39 @@
         <v>1000</v>
       </c>
       <c r="E11">
-        <f>E10+N(C11)-N(D11)</f>
-        <v/>
-      </c>
-      <c r="F11">
+        <f>E10+C11-D11</f>
+        <v/>
+      </c>
+      <c r="F11" s="3">
+        <f>DAYS(A12,A11)</f>
+        <v/>
+      </c>
+      <c r="G11">
+        <f>F11*E11</f>
+        <v/>
+      </c>
+      <c r="I11">
         <f>LOOKUP(A11,Cambi!$A$2:$A$255,Cambi!$B$2:$B$255)</f>
         <v/>
       </c>
-      <c r="G11" s="2">
+      <c r="J11">
+        <f>C11/I11</f>
+        <v/>
+      </c>
+      <c r="L11">
+        <f>L10+J11-K11</f>
+        <v/>
+      </c>
+      <c r="M11" s="3">
+        <f>F11</f>
+        <v/>
+      </c>
+      <c r="N11">
+        <f>M11*L11</f>
+        <v/>
+      </c>
+      <c r="P11" s="2">
         <f>LOOKUP(A11,Cambi!$A$2:$A$255,Cambi!$A$2:$A$255)</f>
-        <v/>
-      </c>
-      <c r="H11">
-        <f>IF(C11="","",C11/F11)</f>
-        <v/>
-      </c>
-      <c r="I11">
-        <f>IF(D11="","",D11/F11)</f>
-        <v/>
-      </c>
-      <c r="J11">
-        <f>J10+N(H11)-N(I11)</f>
-        <v/>
-      </c>
-      <c r="K11">
-        <f>A12-A11</f>
-        <v/>
-      </c>
-      <c r="L11">
-        <f>K11*J11</f>
         <v/>
       </c>
     </row>
@@ -926,35 +983,39 @@
         <v>700</v>
       </c>
       <c r="E12">
-        <f>E11+N(C12)-N(D12)</f>
-        <v/>
-      </c>
-      <c r="F12">
+        <f>E11+C12-D12</f>
+        <v/>
+      </c>
+      <c r="F12" s="3">
+        <f>DAYS(A13,A12)</f>
+        <v/>
+      </c>
+      <c r="G12">
+        <f>F12*E12</f>
+        <v/>
+      </c>
+      <c r="I12">
         <f>LOOKUP(A12,Cambi!$A$2:$A$255,Cambi!$B$2:$B$255)</f>
         <v/>
       </c>
-      <c r="G12" s="2">
+      <c r="K12">
+        <f>D12/I12</f>
+        <v/>
+      </c>
+      <c r="L12">
+        <f>L11+J12-K12</f>
+        <v/>
+      </c>
+      <c r="M12" s="3">
+        <f>F12</f>
+        <v/>
+      </c>
+      <c r="N12">
+        <f>M12*L12</f>
+        <v/>
+      </c>
+      <c r="P12" s="2">
         <f>LOOKUP(A12,Cambi!$A$2:$A$255,Cambi!$A$2:$A$255)</f>
-        <v/>
-      </c>
-      <c r="H12">
-        <f>IF(C12="","",C12/F12)</f>
-        <v/>
-      </c>
-      <c r="I12">
-        <f>IF(D12="","",D12/F12)</f>
-        <v/>
-      </c>
-      <c r="J12">
-        <f>J11+N(H12)-N(I12)</f>
-        <v/>
-      </c>
-      <c r="K12">
-        <f>A13-A12</f>
-        <v/>
-      </c>
-      <c r="L12">
-        <f>K12*J12</f>
         <v/>
       </c>
     </row>
@@ -967,35 +1028,39 @@
         <v>600</v>
       </c>
       <c r="E13">
-        <f>E12+N(C13)-N(D13)</f>
-        <v/>
-      </c>
-      <c r="F13">
+        <f>E12+C13-D13</f>
+        <v/>
+      </c>
+      <c r="F13" s="3">
+        <f>DAYS(A14,A13)</f>
+        <v/>
+      </c>
+      <c r="G13">
+        <f>F13*E13</f>
+        <v/>
+      </c>
+      <c r="I13">
         <f>LOOKUP(A13,Cambi!$A$2:$A$255,Cambi!$B$2:$B$255)</f>
         <v/>
       </c>
-      <c r="G13" s="2">
+      <c r="J13">
+        <f>C13/I13</f>
+        <v/>
+      </c>
+      <c r="L13">
+        <f>L12+J13-K13</f>
+        <v/>
+      </c>
+      <c r="M13" s="3">
+        <f>F13</f>
+        <v/>
+      </c>
+      <c r="N13">
+        <f>M13*L13</f>
+        <v/>
+      </c>
+      <c r="P13" s="2">
         <f>LOOKUP(A13,Cambi!$A$2:$A$255,Cambi!$A$2:$A$255)</f>
-        <v/>
-      </c>
-      <c r="H13">
-        <f>IF(C13="","",C13/F13)</f>
-        <v/>
-      </c>
-      <c r="I13">
-        <f>IF(D13="","",D13/F13)</f>
-        <v/>
-      </c>
-      <c r="J13">
-        <f>J12+N(H13)-N(I13)</f>
-        <v/>
-      </c>
-      <c r="K13">
-        <f>A14-A13</f>
-        <v/>
-      </c>
-      <c r="L13">
-        <f>K13*J13</f>
         <v/>
       </c>
     </row>
@@ -1008,35 +1073,39 @@
         <v>2000</v>
       </c>
       <c r="E14">
-        <f>E13+N(C14)-N(D14)</f>
-        <v/>
-      </c>
-      <c r="F14">
+        <f>E13+C14-D14</f>
+        <v/>
+      </c>
+      <c r="F14" s="3">
+        <f>DAYS(A15,A14)</f>
+        <v/>
+      </c>
+      <c r="G14">
+        <f>F14*E14</f>
+        <v/>
+      </c>
+      <c r="I14">
         <f>LOOKUP(A14,Cambi!$A$2:$A$255,Cambi!$B$2:$B$255)</f>
         <v/>
       </c>
-      <c r="G14" s="2">
+      <c r="J14">
+        <f>C14/I14</f>
+        <v/>
+      </c>
+      <c r="L14">
+        <f>L13+J14-K14</f>
+        <v/>
+      </c>
+      <c r="M14" s="3">
+        <f>F14</f>
+        <v/>
+      </c>
+      <c r="N14">
+        <f>M14*L14</f>
+        <v/>
+      </c>
+      <c r="P14" s="2">
         <f>LOOKUP(A14,Cambi!$A$2:$A$255,Cambi!$A$2:$A$255)</f>
-        <v/>
-      </c>
-      <c r="H14">
-        <f>IF(C14="","",C14/F14)</f>
-        <v/>
-      </c>
-      <c r="I14">
-        <f>IF(D14="","",D14/F14)</f>
-        <v/>
-      </c>
-      <c r="J14">
-        <f>J13+N(H14)-N(I14)</f>
-        <v/>
-      </c>
-      <c r="K14">
-        <f>A15-A14</f>
-        <v/>
-      </c>
-      <c r="L14">
-        <f>K14*J14</f>
         <v/>
       </c>
     </row>
@@ -1049,35 +1118,39 @@
         <v>3510.77</v>
       </c>
       <c r="E15">
-        <f>E14+N(C15)-N(D15)</f>
-        <v/>
-      </c>
-      <c r="F15">
+        <f>E14+C15-D15</f>
+        <v/>
+      </c>
+      <c r="F15" s="3">
+        <f>DAYS(A16,A15)</f>
+        <v/>
+      </c>
+      <c r="G15">
+        <f>F15*E15</f>
+        <v/>
+      </c>
+      <c r="I15">
         <f>LOOKUP(A15,Cambi!$A$2:$A$255,Cambi!$B$2:$B$255)</f>
         <v/>
       </c>
-      <c r="G15" s="2">
+      <c r="K15">
+        <f>D15/I15</f>
+        <v/>
+      </c>
+      <c r="L15">
+        <f>L14+J15-K15</f>
+        <v/>
+      </c>
+      <c r="M15" s="3">
+        <f>F15</f>
+        <v/>
+      </c>
+      <c r="N15">
+        <f>M15*L15</f>
+        <v/>
+      </c>
+      <c r="P15" s="2">
         <f>LOOKUP(A15,Cambi!$A$2:$A$255,Cambi!$A$2:$A$255)</f>
-        <v/>
-      </c>
-      <c r="H15">
-        <f>IF(C15="","",C15/F15)</f>
-        <v/>
-      </c>
-      <c r="I15">
-        <f>IF(D15="","",D15/F15)</f>
-        <v/>
-      </c>
-      <c r="J15">
-        <f>J14+N(H15)-N(I15)</f>
-        <v/>
-      </c>
-      <c r="K15">
-        <f>A16-A15</f>
-        <v/>
-      </c>
-      <c r="L15">
-        <f>K15*J15</f>
         <v/>
       </c>
     </row>
@@ -1090,35 +1163,39 @@
         <v>597.6</v>
       </c>
       <c r="E16">
-        <f>E15+N(C16)-N(D16)</f>
-        <v/>
-      </c>
-      <c r="F16">
+        <f>E15+C16-D16</f>
+        <v/>
+      </c>
+      <c r="F16" s="3">
+        <f>DAYS(A17,A16)</f>
+        <v/>
+      </c>
+      <c r="G16">
+        <f>F16*E16</f>
+        <v/>
+      </c>
+      <c r="I16">
         <f>LOOKUP(A16,Cambi!$A$2:$A$255,Cambi!$B$2:$B$255)</f>
         <v/>
       </c>
-      <c r="G16" s="2">
+      <c r="K16">
+        <f>D16/I16</f>
+        <v/>
+      </c>
+      <c r="L16">
+        <f>L15+J16-K16</f>
+        <v/>
+      </c>
+      <c r="M16" s="3">
+        <f>F16</f>
+        <v/>
+      </c>
+      <c r="N16">
+        <f>M16*L16</f>
+        <v/>
+      </c>
+      <c r="P16" s="2">
         <f>LOOKUP(A16,Cambi!$A$2:$A$255,Cambi!$A$2:$A$255)</f>
-        <v/>
-      </c>
-      <c r="H16">
-        <f>IF(C16="","",C16/F16)</f>
-        <v/>
-      </c>
-      <c r="I16">
-        <f>IF(D16="","",D16/F16)</f>
-        <v/>
-      </c>
-      <c r="J16">
-        <f>J15+N(H16)-N(I16)</f>
-        <v/>
-      </c>
-      <c r="K16">
-        <f>A17-A16</f>
-        <v/>
-      </c>
-      <c r="L16">
-        <f>K16*J16</f>
         <v/>
       </c>
     </row>
@@ -1131,35 +1208,39 @@
         <v>1000</v>
       </c>
       <c r="E17">
-        <f>E16+N(C17)-N(D17)</f>
-        <v/>
-      </c>
-      <c r="F17">
+        <f>E16+C17-D17</f>
+        <v/>
+      </c>
+      <c r="F17" s="3">
+        <f>DAYS(A18,A17)</f>
+        <v/>
+      </c>
+      <c r="G17">
+        <f>F17*E17</f>
+        <v/>
+      </c>
+      <c r="I17">
         <f>LOOKUP(A17,Cambi!$A$2:$A$255,Cambi!$B$2:$B$255)</f>
         <v/>
       </c>
-      <c r="G17" s="2">
+      <c r="J17">
+        <f>C17/I17</f>
+        <v/>
+      </c>
+      <c r="L17">
+        <f>L16+J17-K17</f>
+        <v/>
+      </c>
+      <c r="M17" s="3">
+        <f>F17</f>
+        <v/>
+      </c>
+      <c r="N17">
+        <f>M17*L17</f>
+        <v/>
+      </c>
+      <c r="P17" s="2">
         <f>LOOKUP(A17,Cambi!$A$2:$A$255,Cambi!$A$2:$A$255)</f>
-        <v/>
-      </c>
-      <c r="H17">
-        <f>IF(C17="","",C17/F17)</f>
-        <v/>
-      </c>
-      <c r="I17">
-        <f>IF(D17="","",D17/F17)</f>
-        <v/>
-      </c>
-      <c r="J17">
-        <f>J16+N(H17)-N(I17)</f>
-        <v/>
-      </c>
-      <c r="K17">
-        <f>A18-A17</f>
-        <v/>
-      </c>
-      <c r="L17">
-        <f>K17*J17</f>
         <v/>
       </c>
     </row>
@@ -1172,35 +1253,39 @@
         <v>600</v>
       </c>
       <c r="E18">
-        <f>E17+N(C18)-N(D18)</f>
-        <v/>
-      </c>
-      <c r="F18">
+        <f>E17+C18-D18</f>
+        <v/>
+      </c>
+      <c r="F18" s="3">
+        <f>DAYS(A19,A18)</f>
+        <v/>
+      </c>
+      <c r="G18">
+        <f>F18*E18</f>
+        <v/>
+      </c>
+      <c r="I18">
         <f>LOOKUP(A18,Cambi!$A$2:$A$255,Cambi!$B$2:$B$255)</f>
         <v/>
       </c>
-      <c r="G18" s="2">
+      <c r="J18">
+        <f>C18/I18</f>
+        <v/>
+      </c>
+      <c r="L18">
+        <f>L17+J18-K18</f>
+        <v/>
+      </c>
+      <c r="M18" s="3">
+        <f>F18</f>
+        <v/>
+      </c>
+      <c r="N18">
+        <f>M18*L18</f>
+        <v/>
+      </c>
+      <c r="P18" s="2">
         <f>LOOKUP(A18,Cambi!$A$2:$A$255,Cambi!$A$2:$A$255)</f>
-        <v/>
-      </c>
-      <c r="H18">
-        <f>IF(C18="","",C18/F18)</f>
-        <v/>
-      </c>
-      <c r="I18">
-        <f>IF(D18="","",D18/F18)</f>
-        <v/>
-      </c>
-      <c r="J18">
-        <f>J17+N(H18)-N(I18)</f>
-        <v/>
-      </c>
-      <c r="K18">
-        <f>A19-A18</f>
-        <v/>
-      </c>
-      <c r="L18">
-        <f>K18*J18</f>
         <v/>
       </c>
     </row>
@@ -1213,35 +1298,39 @@
         <v>1000</v>
       </c>
       <c r="E19">
-        <f>E18+N(C19)-N(D19)</f>
-        <v/>
-      </c>
-      <c r="F19">
+        <f>E18+C19-D19</f>
+        <v/>
+      </c>
+      <c r="F19" s="3">
+        <f>DAYS(A20,A19)</f>
+        <v/>
+      </c>
+      <c r="G19">
+        <f>F19*E19</f>
+        <v/>
+      </c>
+      <c r="I19">
         <f>LOOKUP(A19,Cambi!$A$2:$A$255,Cambi!$B$2:$B$255)</f>
         <v/>
       </c>
-      <c r="G19" s="2">
+      <c r="J19">
+        <f>C19/I19</f>
+        <v/>
+      </c>
+      <c r="L19">
+        <f>L18+J19-K19</f>
+        <v/>
+      </c>
+      <c r="M19" s="3">
+        <f>F19</f>
+        <v/>
+      </c>
+      <c r="N19">
+        <f>M19*L19</f>
+        <v/>
+      </c>
+      <c r="P19" s="2">
         <f>LOOKUP(A19,Cambi!$A$2:$A$255,Cambi!$A$2:$A$255)</f>
-        <v/>
-      </c>
-      <c r="H19">
-        <f>IF(C19="","",C19/F19)</f>
-        <v/>
-      </c>
-      <c r="I19">
-        <f>IF(D19="","",D19/F19)</f>
-        <v/>
-      </c>
-      <c r="J19">
-        <f>J18+N(H19)-N(I19)</f>
-        <v/>
-      </c>
-      <c r="K19">
-        <f>A20-A19</f>
-        <v/>
-      </c>
-      <c r="L19">
-        <f>K19*J19</f>
         <v/>
       </c>
     </row>
@@ -1254,35 +1343,39 @@
         <v>600</v>
       </c>
       <c r="E20">
-        <f>E19+N(C20)-N(D20)</f>
-        <v/>
-      </c>
-      <c r="F20">
+        <f>E19+C20-D20</f>
+        <v/>
+      </c>
+      <c r="F20" s="3">
+        <f>DAYS(A21,A20)</f>
+        <v/>
+      </c>
+      <c r="G20">
+        <f>F20*E20</f>
+        <v/>
+      </c>
+      <c r="I20">
         <f>LOOKUP(A20,Cambi!$A$2:$A$255,Cambi!$B$2:$B$255)</f>
         <v/>
       </c>
-      <c r="G20" s="2">
+      <c r="J20">
+        <f>C20/I20</f>
+        <v/>
+      </c>
+      <c r="L20">
+        <f>L19+J20-K20</f>
+        <v/>
+      </c>
+      <c r="M20" s="3">
+        <f>F20</f>
+        <v/>
+      </c>
+      <c r="N20">
+        <f>M20*L20</f>
+        <v/>
+      </c>
+      <c r="P20" s="2">
         <f>LOOKUP(A20,Cambi!$A$2:$A$255,Cambi!$A$2:$A$255)</f>
-        <v/>
-      </c>
-      <c r="H20">
-        <f>IF(C20="","",C20/F20)</f>
-        <v/>
-      </c>
-      <c r="I20">
-        <f>IF(D20="","",D20/F20)</f>
-        <v/>
-      </c>
-      <c r="J20">
-        <f>J19+N(H20)-N(I20)</f>
-        <v/>
-      </c>
-      <c r="K20">
-        <f>A21-A20</f>
-        <v/>
-      </c>
-      <c r="L20">
-        <f>K20*J20</f>
         <v/>
       </c>
     </row>
@@ -1295,35 +1388,39 @@
         <v>10000</v>
       </c>
       <c r="E21">
-        <f>E20+N(C21)-N(D21)</f>
-        <v/>
-      </c>
-      <c r="F21">
+        <f>E20+C21-D21</f>
+        <v/>
+      </c>
+      <c r="F21" s="3">
+        <f>DAYS(A22,A21)</f>
+        <v/>
+      </c>
+      <c r="G21">
+        <f>F21*E21</f>
+        <v/>
+      </c>
+      <c r="I21">
         <f>LOOKUP(A21,Cambi!$A$2:$A$255,Cambi!$B$2:$B$255)</f>
         <v/>
       </c>
-      <c r="G21" s="2">
+      <c r="J21">
+        <f>C21/I21</f>
+        <v/>
+      </c>
+      <c r="L21">
+        <f>L20+J21-K21</f>
+        <v/>
+      </c>
+      <c r="M21" s="3">
+        <f>F21</f>
+        <v/>
+      </c>
+      <c r="N21">
+        <f>M21*L21</f>
+        <v/>
+      </c>
+      <c r="P21" s="2">
         <f>LOOKUP(A21,Cambi!$A$2:$A$255,Cambi!$A$2:$A$255)</f>
-        <v/>
-      </c>
-      <c r="H21">
-        <f>IF(C21="","",C21/F21)</f>
-        <v/>
-      </c>
-      <c r="I21">
-        <f>IF(D21="","",D21/F21)</f>
-        <v/>
-      </c>
-      <c r="J21">
-        <f>J20+N(H21)-N(I21)</f>
-        <v/>
-      </c>
-      <c r="K21">
-        <f>A22-A21</f>
-        <v/>
-      </c>
-      <c r="L21">
-        <f>K21*J21</f>
         <v/>
       </c>
     </row>
@@ -1336,35 +1433,39 @@
         <v>11976</v>
       </c>
       <c r="E22">
-        <f>E21+N(C22)-N(D22)</f>
-        <v/>
-      </c>
-      <c r="F22">
+        <f>E21+C22-D22</f>
+        <v/>
+      </c>
+      <c r="F22" s="3">
+        <f>DAYS(A23,A22)</f>
+        <v/>
+      </c>
+      <c r="G22">
+        <f>F22*E22</f>
+        <v/>
+      </c>
+      <c r="I22">
         <f>LOOKUP(A22,Cambi!$A$2:$A$255,Cambi!$B$2:$B$255)</f>
         <v/>
       </c>
-      <c r="G22" s="2">
+      <c r="K22">
+        <f>D22/I22</f>
+        <v/>
+      </c>
+      <c r="L22">
+        <f>L21+J22-K22</f>
+        <v/>
+      </c>
+      <c r="M22" s="3">
+        <f>F22</f>
+        <v/>
+      </c>
+      <c r="N22">
+        <f>M22*L22</f>
+        <v/>
+      </c>
+      <c r="P22" s="2">
         <f>LOOKUP(A22,Cambi!$A$2:$A$255,Cambi!$A$2:$A$255)</f>
-        <v/>
-      </c>
-      <c r="H22">
-        <f>IF(C22="","",C22/F22)</f>
-        <v/>
-      </c>
-      <c r="I22">
-        <f>IF(D22="","",D22/F22)</f>
-        <v/>
-      </c>
-      <c r="J22">
-        <f>J21+N(H22)-N(I22)</f>
-        <v/>
-      </c>
-      <c r="K22">
-        <f>A23-A22</f>
-        <v/>
-      </c>
-      <c r="L22">
-        <f>K22*J22</f>
         <v/>
       </c>
     </row>
@@ -1377,35 +1478,39 @@
         <v>1000</v>
       </c>
       <c r="E23">
-        <f>E22+N(C23)-N(D23)</f>
-        <v/>
-      </c>
-      <c r="F23">
+        <f>E22+C23-D23</f>
+        <v/>
+      </c>
+      <c r="F23" s="3">
+        <f>DAYS(A24,A23)</f>
+        <v/>
+      </c>
+      <c r="G23">
+        <f>F23*E23</f>
+        <v/>
+      </c>
+      <c r="I23">
         <f>LOOKUP(A23,Cambi!$A$2:$A$255,Cambi!$B$2:$B$255)</f>
         <v/>
       </c>
-      <c r="G23" s="2">
+      <c r="J23">
+        <f>C23/I23</f>
+        <v/>
+      </c>
+      <c r="L23">
+        <f>L22+J23-K23</f>
+        <v/>
+      </c>
+      <c r="M23" s="3">
+        <f>F23</f>
+        <v/>
+      </c>
+      <c r="N23">
+        <f>M23*L23</f>
+        <v/>
+      </c>
+      <c r="P23" s="2">
         <f>LOOKUP(A23,Cambi!$A$2:$A$255,Cambi!$A$2:$A$255)</f>
-        <v/>
-      </c>
-      <c r="H23">
-        <f>IF(C23="","",C23/F23)</f>
-        <v/>
-      </c>
-      <c r="I23">
-        <f>IF(D23="","",D23/F23)</f>
-        <v/>
-      </c>
-      <c r="J23">
-        <f>J22+N(H23)-N(I23)</f>
-        <v/>
-      </c>
-      <c r="K23">
-        <f>A24-A23</f>
-        <v/>
-      </c>
-      <c r="L23">
-        <f>K23*J23</f>
         <v/>
       </c>
     </row>
@@ -1418,35 +1523,39 @@
         <v>600</v>
       </c>
       <c r="E24">
-        <f>E23+N(C24)-N(D24)</f>
-        <v/>
-      </c>
-      <c r="F24">
+        <f>E23+C24-D24</f>
+        <v/>
+      </c>
+      <c r="F24" s="3">
+        <f>DAYS(A25,A24)</f>
+        <v/>
+      </c>
+      <c r="G24">
+        <f>F24*E24</f>
+        <v/>
+      </c>
+      <c r="I24">
         <f>LOOKUP(A24,Cambi!$A$2:$A$255,Cambi!$B$2:$B$255)</f>
         <v/>
       </c>
-      <c r="G24" s="2">
+      <c r="J24">
+        <f>C24/I24</f>
+        <v/>
+      </c>
+      <c r="L24">
+        <f>L23+J24-K24</f>
+        <v/>
+      </c>
+      <c r="M24" s="3">
+        <f>F24</f>
+        <v/>
+      </c>
+      <c r="N24">
+        <f>M24*L24</f>
+        <v/>
+      </c>
+      <c r="P24" s="2">
         <f>LOOKUP(A24,Cambi!$A$2:$A$255,Cambi!$A$2:$A$255)</f>
-        <v/>
-      </c>
-      <c r="H24">
-        <f>IF(C24="","",C24/F24)</f>
-        <v/>
-      </c>
-      <c r="I24">
-        <f>IF(D24="","",D24/F24)</f>
-        <v/>
-      </c>
-      <c r="J24">
-        <f>J23+N(H24)-N(I24)</f>
-        <v/>
-      </c>
-      <c r="K24">
-        <f>A25-A24</f>
-        <v/>
-      </c>
-      <c r="L24">
-        <f>K24*J24</f>
         <v/>
       </c>
     </row>
@@ -1459,35 +1568,39 @@
         <v>1000</v>
       </c>
       <c r="E25">
-        <f>E24+N(C25)-N(D25)</f>
-        <v/>
-      </c>
-      <c r="F25">
+        <f>E24+C25-D25</f>
+        <v/>
+      </c>
+      <c r="F25" s="3">
+        <f>DAYS(A26,A25)</f>
+        <v/>
+      </c>
+      <c r="G25">
+        <f>F25*E25</f>
+        <v/>
+      </c>
+      <c r="I25">
         <f>LOOKUP(A25,Cambi!$A$2:$A$255,Cambi!$B$2:$B$255)</f>
         <v/>
       </c>
-      <c r="G25" s="2">
+      <c r="J25">
+        <f>C25/I25</f>
+        <v/>
+      </c>
+      <c r="L25">
+        <f>L24+J25-K25</f>
+        <v/>
+      </c>
+      <c r="M25" s="3">
+        <f>F25</f>
+        <v/>
+      </c>
+      <c r="N25">
+        <f>M25*L25</f>
+        <v/>
+      </c>
+      <c r="P25" s="2">
         <f>LOOKUP(A25,Cambi!$A$2:$A$255,Cambi!$A$2:$A$255)</f>
-        <v/>
-      </c>
-      <c r="H25">
-        <f>IF(C25="","",C25/F25)</f>
-        <v/>
-      </c>
-      <c r="I25">
-        <f>IF(D25="","",D25/F25)</f>
-        <v/>
-      </c>
-      <c r="J25">
-        <f>J24+N(H25)-N(I25)</f>
-        <v/>
-      </c>
-      <c r="K25">
-        <f>A26-A25</f>
-        <v/>
-      </c>
-      <c r="L25">
-        <f>K25*J25</f>
         <v/>
       </c>
     </row>
@@ -1500,35 +1613,39 @@
         <v>600</v>
       </c>
       <c r="E26">
-        <f>E25+N(C26)-N(D26)</f>
-        <v/>
-      </c>
-      <c r="F26">
+        <f>E25+C26-D26</f>
+        <v/>
+      </c>
+      <c r="F26" s="3">
+        <f>DAYS(A27,A26)</f>
+        <v/>
+      </c>
+      <c r="G26">
+        <f>F26*E26</f>
+        <v/>
+      </c>
+      <c r="I26">
         <f>LOOKUP(A26,Cambi!$A$2:$A$255,Cambi!$B$2:$B$255)</f>
         <v/>
       </c>
-      <c r="G26" s="2">
+      <c r="J26">
+        <f>C26/I26</f>
+        <v/>
+      </c>
+      <c r="L26">
+        <f>L25+J26-K26</f>
+        <v/>
+      </c>
+      <c r="M26" s="3">
+        <f>F26</f>
+        <v/>
+      </c>
+      <c r="N26">
+        <f>M26*L26</f>
+        <v/>
+      </c>
+      <c r="P26" s="2">
         <f>LOOKUP(A26,Cambi!$A$2:$A$255,Cambi!$A$2:$A$255)</f>
-        <v/>
-      </c>
-      <c r="H26">
-        <f>IF(C26="","",C26/F26)</f>
-        <v/>
-      </c>
-      <c r="I26">
-        <f>IF(D26="","",D26/F26)</f>
-        <v/>
-      </c>
-      <c r="J26">
-        <f>J25+N(H26)-N(I26)</f>
-        <v/>
-      </c>
-      <c r="K26">
-        <f>A27-A26</f>
-        <v/>
-      </c>
-      <c r="L26">
-        <f>K26*J26</f>
         <v/>
       </c>
     </row>
@@ -1541,35 +1658,39 @@
         <v>3000</v>
       </c>
       <c r="E27">
-        <f>E26+N(C27)-N(D27)</f>
-        <v/>
-      </c>
-      <c r="F27">
+        <f>E26+C27-D27</f>
+        <v/>
+      </c>
+      <c r="F27" s="3">
+        <f>DAYS(A28,A27)</f>
+        <v/>
+      </c>
+      <c r="G27">
+        <f>F27*E27</f>
+        <v/>
+      </c>
+      <c r="I27">
         <f>LOOKUP(A27,Cambi!$A$2:$A$255,Cambi!$B$2:$B$255)</f>
         <v/>
       </c>
-      <c r="G27" s="2">
+      <c r="K27">
+        <f>D27/I27</f>
+        <v/>
+      </c>
+      <c r="L27">
+        <f>L26+J27-K27</f>
+        <v/>
+      </c>
+      <c r="M27" s="3">
+        <f>F27</f>
+        <v/>
+      </c>
+      <c r="N27">
+        <f>M27*L27</f>
+        <v/>
+      </c>
+      <c r="P27" s="2">
         <f>LOOKUP(A27,Cambi!$A$2:$A$255,Cambi!$A$2:$A$255)</f>
-        <v/>
-      </c>
-      <c r="H27">
-        <f>IF(C27="","",C27/F27)</f>
-        <v/>
-      </c>
-      <c r="I27">
-        <f>IF(D27="","",D27/F27)</f>
-        <v/>
-      </c>
-      <c r="J27">
-        <f>J26+N(H27)-N(I27)</f>
-        <v/>
-      </c>
-      <c r="K27">
-        <f>A28-A27</f>
-        <v/>
-      </c>
-      <c r="L27">
-        <f>K27*J27</f>
         <v/>
       </c>
     </row>
@@ -1582,35 +1703,39 @@
         <v>1480</v>
       </c>
       <c r="E28">
-        <f>E27+N(C28)-N(D28)</f>
-        <v/>
-      </c>
-      <c r="F28">
+        <f>E27+C28-D28</f>
+        <v/>
+      </c>
+      <c r="F28" s="3">
+        <f>DAYS(A29,A28)</f>
+        <v/>
+      </c>
+      <c r="G28">
+        <f>F28*E28</f>
+        <v/>
+      </c>
+      <c r="I28">
         <f>LOOKUP(A28,Cambi!$A$2:$A$255,Cambi!$B$2:$B$255)</f>
         <v/>
       </c>
-      <c r="G28" s="2">
+      <c r="K28">
+        <f>D28/I28</f>
+        <v/>
+      </c>
+      <c r="L28">
+        <f>L27+J28-K28</f>
+        <v/>
+      </c>
+      <c r="M28" s="3">
+        <f>F28</f>
+        <v/>
+      </c>
+      <c r="N28">
+        <f>M28*L28</f>
+        <v/>
+      </c>
+      <c r="P28" s="2">
         <f>LOOKUP(A28,Cambi!$A$2:$A$255,Cambi!$A$2:$A$255)</f>
-        <v/>
-      </c>
-      <c r="H28">
-        <f>IF(C28="","",C28/F28)</f>
-        <v/>
-      </c>
-      <c r="I28">
-        <f>IF(D28="","",D28/F28)</f>
-        <v/>
-      </c>
-      <c r="J28">
-        <f>J27+N(H28)-N(I28)</f>
-        <v/>
-      </c>
-      <c r="K28">
-        <f>A29-A28</f>
-        <v/>
-      </c>
-      <c r="L28">
-        <f>K28*J28</f>
         <v/>
       </c>
     </row>
@@ -1623,35 +1748,39 @@
         <v>600</v>
       </c>
       <c r="E29">
-        <f>E28+N(C29)-N(D29)</f>
-        <v/>
-      </c>
-      <c r="F29">
+        <f>E28+C29-D29</f>
+        <v/>
+      </c>
+      <c r="F29" s="3">
+        <f>DAYS(A30,A29)</f>
+        <v/>
+      </c>
+      <c r="G29">
+        <f>F29*E29</f>
+        <v/>
+      </c>
+      <c r="I29">
         <f>LOOKUP(A29,Cambi!$A$2:$A$255,Cambi!$B$2:$B$255)</f>
         <v/>
       </c>
-      <c r="G29" s="2">
+      <c r="J29">
+        <f>C29/I29</f>
+        <v/>
+      </c>
+      <c r="L29">
+        <f>L28+J29-K29</f>
+        <v/>
+      </c>
+      <c r="M29" s="3">
+        <f>F29</f>
+        <v/>
+      </c>
+      <c r="N29">
+        <f>M29*L29</f>
+        <v/>
+      </c>
+      <c r="P29" s="2">
         <f>LOOKUP(A29,Cambi!$A$2:$A$255,Cambi!$A$2:$A$255)</f>
-        <v/>
-      </c>
-      <c r="H29">
-        <f>IF(C29="","",C29/F29)</f>
-        <v/>
-      </c>
-      <c r="I29">
-        <f>IF(D29="","",D29/F29)</f>
-        <v/>
-      </c>
-      <c r="J29">
-        <f>J28+N(H29)-N(I29)</f>
-        <v/>
-      </c>
-      <c r="K29">
-        <f>A30-A29</f>
-        <v/>
-      </c>
-      <c r="L29">
-        <f>K29*J29</f>
         <v/>
       </c>
     </row>
@@ -1664,35 +1793,39 @@
         <v>4000</v>
       </c>
       <c r="E30">
-        <f>E29+N(C30)-N(D30)</f>
-        <v/>
-      </c>
-      <c r="F30">
+        <f>E29+C30-D30</f>
+        <v/>
+      </c>
+      <c r="F30" s="3">
+        <f>DAYS(A31,A30)</f>
+        <v/>
+      </c>
+      <c r="G30">
+        <f>F30*E30</f>
+        <v/>
+      </c>
+      <c r="I30">
         <f>LOOKUP(A30,Cambi!$A$2:$A$255,Cambi!$B$2:$B$255)</f>
         <v/>
       </c>
-      <c r="G30" s="2">
+      <c r="J30">
+        <f>C30/I30</f>
+        <v/>
+      </c>
+      <c r="L30">
+        <f>L29+J30-K30</f>
+        <v/>
+      </c>
+      <c r="M30" s="3">
+        <f>F30</f>
+        <v/>
+      </c>
+      <c r="N30">
+        <f>M30*L30</f>
+        <v/>
+      </c>
+      <c r="P30" s="2">
         <f>LOOKUP(A30,Cambi!$A$2:$A$255,Cambi!$A$2:$A$255)</f>
-        <v/>
-      </c>
-      <c r="H30">
-        <f>IF(C30="","",C30/F30)</f>
-        <v/>
-      </c>
-      <c r="I30">
-        <f>IF(D30="","",D30/F30)</f>
-        <v/>
-      </c>
-      <c r="J30">
-        <f>J29+N(H30)-N(I30)</f>
-        <v/>
-      </c>
-      <c r="K30">
-        <f>A31-A30</f>
-        <v/>
-      </c>
-      <c r="L30">
-        <f>K30*J30</f>
         <v/>
       </c>
     </row>
@@ -1705,35 +1838,39 @@
         <v>4941.4</v>
       </c>
       <c r="E31">
-        <f>E30+N(C31)-N(D31)</f>
-        <v/>
-      </c>
-      <c r="F31">
+        <f>E30+C31-D31</f>
+        <v/>
+      </c>
+      <c r="F31" s="3">
+        <f>DAYS(A32,A31)</f>
+        <v/>
+      </c>
+      <c r="G31">
+        <f>F31*E31</f>
+        <v/>
+      </c>
+      <c r="I31">
         <f>LOOKUP(A31,Cambi!$A$2:$A$255,Cambi!$B$2:$B$255)</f>
         <v/>
       </c>
-      <c r="G31" s="2">
+      <c r="K31">
+        <f>D31/I31</f>
+        <v/>
+      </c>
+      <c r="L31">
+        <f>L30+J31-K31</f>
+        <v/>
+      </c>
+      <c r="M31" s="3">
+        <f>F31</f>
+        <v/>
+      </c>
+      <c r="N31">
+        <f>M31*L31</f>
+        <v/>
+      </c>
+      <c r="P31" s="2">
         <f>LOOKUP(A31,Cambi!$A$2:$A$255,Cambi!$A$2:$A$255)</f>
-        <v/>
-      </c>
-      <c r="H31">
-        <f>IF(C31="","",C31/F31)</f>
-        <v/>
-      </c>
-      <c r="I31">
-        <f>IF(D31="","",D31/F31)</f>
-        <v/>
-      </c>
-      <c r="J31">
-        <f>J30+N(H31)-N(I31)</f>
-        <v/>
-      </c>
-      <c r="K31">
-        <f>A32-A31</f>
-        <v/>
-      </c>
-      <c r="L31">
-        <f>K31*J31</f>
         <v/>
       </c>
     </row>
@@ -1746,35 +1883,39 @@
         <v>1000</v>
       </c>
       <c r="E32">
-        <f>E31+N(C32)-N(D32)</f>
-        <v/>
-      </c>
-      <c r="F32">
+        <f>E31+C32-D32</f>
+        <v/>
+      </c>
+      <c r="F32" s="3">
+        <f>DAYS(A33,A32)</f>
+        <v/>
+      </c>
+      <c r="G32">
+        <f>F32*E32</f>
+        <v/>
+      </c>
+      <c r="I32">
         <f>LOOKUP(A32,Cambi!$A$2:$A$255,Cambi!$B$2:$B$255)</f>
         <v/>
       </c>
-      <c r="G32" s="2">
+      <c r="J32">
+        <f>C32/I32</f>
+        <v/>
+      </c>
+      <c r="L32">
+        <f>L31+J32-K32</f>
+        <v/>
+      </c>
+      <c r="M32" s="3">
+        <f>F32</f>
+        <v/>
+      </c>
+      <c r="N32">
+        <f>M32*L32</f>
+        <v/>
+      </c>
+      <c r="P32" s="2">
         <f>LOOKUP(A32,Cambi!$A$2:$A$255,Cambi!$A$2:$A$255)</f>
-        <v/>
-      </c>
-      <c r="H32">
-        <f>IF(C32="","",C32/F32)</f>
-        <v/>
-      </c>
-      <c r="I32">
-        <f>IF(D32="","",D32/F32)</f>
-        <v/>
-      </c>
-      <c r="J32">
-        <f>J31+N(H32)-N(I32)</f>
-        <v/>
-      </c>
-      <c r="K32">
-        <f>A33-A32</f>
-        <v/>
-      </c>
-      <c r="L32">
-        <f>K32*J32</f>
         <v/>
       </c>
     </row>
@@ -1787,35 +1928,39 @@
         <v>180</v>
       </c>
       <c r="E33">
-        <f>E32+N(C33)-N(D33)</f>
-        <v/>
-      </c>
-      <c r="F33">
+        <f>E32+C33-D33</f>
+        <v/>
+      </c>
+      <c r="F33" s="3">
+        <f>DAYS(A34,A33)</f>
+        <v/>
+      </c>
+      <c r="G33">
+        <f>F33*E33</f>
+        <v/>
+      </c>
+      <c r="I33">
         <f>LOOKUP(A33,Cambi!$A$2:$A$255,Cambi!$B$2:$B$255)</f>
         <v/>
       </c>
-      <c r="G33" s="2">
+      <c r="K33">
+        <f>D33/I33</f>
+        <v/>
+      </c>
+      <c r="L33">
+        <f>L32+J33-K33</f>
+        <v/>
+      </c>
+      <c r="M33" s="3">
+        <f>F33</f>
+        <v/>
+      </c>
+      <c r="N33">
+        <f>M33*L33</f>
+        <v/>
+      </c>
+      <c r="P33" s="2">
         <f>LOOKUP(A33,Cambi!$A$2:$A$255,Cambi!$A$2:$A$255)</f>
-        <v/>
-      </c>
-      <c r="H33">
-        <f>IF(C33="","",C33/F33)</f>
-        <v/>
-      </c>
-      <c r="I33">
-        <f>IF(D33="","",D33/F33)</f>
-        <v/>
-      </c>
-      <c r="J33">
-        <f>J32+N(H33)-N(I33)</f>
-        <v/>
-      </c>
-      <c r="K33">
-        <f>A34-A33</f>
-        <v/>
-      </c>
-      <c r="L33">
-        <f>K33*J33</f>
         <v/>
       </c>
     </row>
@@ -1828,35 +1973,39 @@
         <v>600</v>
       </c>
       <c r="E34">
-        <f>E33+N(C34)-N(D34)</f>
-        <v/>
-      </c>
-      <c r="F34">
+        <f>E33+C34-D34</f>
+        <v/>
+      </c>
+      <c r="F34" s="3">
+        <f>DAYS(A35,A34)</f>
+        <v/>
+      </c>
+      <c r="G34">
+        <f>F34*E34</f>
+        <v/>
+      </c>
+      <c r="I34">
         <f>LOOKUP(A34,Cambi!$A$2:$A$255,Cambi!$B$2:$B$255)</f>
         <v/>
       </c>
-      <c r="G34" s="2">
+      <c r="J34">
+        <f>C34/I34</f>
+        <v/>
+      </c>
+      <c r="L34">
+        <f>L33+J34-K34</f>
+        <v/>
+      </c>
+      <c r="M34" s="3">
+        <f>F34</f>
+        <v/>
+      </c>
+      <c r="N34">
+        <f>M34*L34</f>
+        <v/>
+      </c>
+      <c r="P34" s="2">
         <f>LOOKUP(A34,Cambi!$A$2:$A$255,Cambi!$A$2:$A$255)</f>
-        <v/>
-      </c>
-      <c r="H34">
-        <f>IF(C34="","",C34/F34)</f>
-        <v/>
-      </c>
-      <c r="I34">
-        <f>IF(D34="","",D34/F34)</f>
-        <v/>
-      </c>
-      <c r="J34">
-        <f>J33+N(H34)-N(I34)</f>
-        <v/>
-      </c>
-      <c r="K34">
-        <f>A35-A34</f>
-        <v/>
-      </c>
-      <c r="L34">
-        <f>K34*J34</f>
         <v/>
       </c>
     </row>
@@ -1869,35 +2018,39 @@
         <v>1000</v>
       </c>
       <c r="E35">
-        <f>E34+N(C35)-N(D35)</f>
-        <v/>
-      </c>
-      <c r="F35">
+        <f>E34+C35-D35</f>
+        <v/>
+      </c>
+      <c r="F35" s="3">
+        <f>DAYS(A36,A35)</f>
+        <v/>
+      </c>
+      <c r="G35">
+        <f>F35*E35</f>
+        <v/>
+      </c>
+      <c r="I35">
         <f>LOOKUP(A35,Cambi!$A$2:$A$255,Cambi!$B$2:$B$255)</f>
         <v/>
       </c>
-      <c r="G35" s="2">
+      <c r="J35">
+        <f>C35/I35</f>
+        <v/>
+      </c>
+      <c r="L35">
+        <f>L34+J35-K35</f>
+        <v/>
+      </c>
+      <c r="M35" s="3">
+        <f>F35</f>
+        <v/>
+      </c>
+      <c r="N35">
+        <f>M35*L35</f>
+        <v/>
+      </c>
+      <c r="P35" s="2">
         <f>LOOKUP(A35,Cambi!$A$2:$A$255,Cambi!$A$2:$A$255)</f>
-        <v/>
-      </c>
-      <c r="H35">
-        <f>IF(C35="","",C35/F35)</f>
-        <v/>
-      </c>
-      <c r="I35">
-        <f>IF(D35="","",D35/F35)</f>
-        <v/>
-      </c>
-      <c r="J35">
-        <f>J34+N(H35)-N(I35)</f>
-        <v/>
-      </c>
-      <c r="K35">
-        <f>A36-A35</f>
-        <v/>
-      </c>
-      <c r="L35">
-        <f>K35*J35</f>
         <v/>
       </c>
     </row>
@@ -1910,35 +2063,39 @@
         <v>600</v>
       </c>
       <c r="E36">
-        <f>E35+N(C36)-N(D36)</f>
-        <v/>
-      </c>
-      <c r="F36">
+        <f>E35+C36-D36</f>
+        <v/>
+      </c>
+      <c r="F36" s="3">
+        <f>DAYS(A37,A36)</f>
+        <v/>
+      </c>
+      <c r="G36">
+        <f>F36*E36</f>
+        <v/>
+      </c>
+      <c r="I36">
         <f>LOOKUP(A36,Cambi!$A$2:$A$255,Cambi!$B$2:$B$255)</f>
         <v/>
       </c>
-      <c r="G36" s="2">
+      <c r="J36">
+        <f>C36/I36</f>
+        <v/>
+      </c>
+      <c r="L36">
+        <f>L35+J36-K36</f>
+        <v/>
+      </c>
+      <c r="M36" s="3">
+        <f>F36</f>
+        <v/>
+      </c>
+      <c r="N36">
+        <f>M36*L36</f>
+        <v/>
+      </c>
+      <c r="P36" s="2">
         <f>LOOKUP(A36,Cambi!$A$2:$A$255,Cambi!$A$2:$A$255)</f>
-        <v/>
-      </c>
-      <c r="H36">
-        <f>IF(C36="","",C36/F36)</f>
-        <v/>
-      </c>
-      <c r="I36">
-        <f>IF(D36="","",D36/F36)</f>
-        <v/>
-      </c>
-      <c r="J36">
-        <f>J35+N(H36)-N(I36)</f>
-        <v/>
-      </c>
-      <c r="K36">
-        <f>A37-A36</f>
-        <v/>
-      </c>
-      <c r="L36">
-        <f>K36*J36</f>
         <v/>
       </c>
     </row>
@@ -1951,35 +2108,39 @@
         <v>2000</v>
       </c>
       <c r="E37">
-        <f>E36+N(C37)-N(D37)</f>
-        <v/>
-      </c>
-      <c r="F37">
+        <f>E36+C37-D37</f>
+        <v/>
+      </c>
+      <c r="F37" s="3">
+        <f>DAYS(A38,A37)</f>
+        <v/>
+      </c>
+      <c r="G37">
+        <f>F37*E37</f>
+        <v/>
+      </c>
+      <c r="I37">
         <f>LOOKUP(A37,Cambi!$A$2:$A$255,Cambi!$B$2:$B$255)</f>
         <v/>
       </c>
-      <c r="G37" s="2">
+      <c r="K37">
+        <f>D37/I37</f>
+        <v/>
+      </c>
+      <c r="L37">
+        <f>L36+J37-K37</f>
+        <v/>
+      </c>
+      <c r="M37" s="3">
+        <f>F37</f>
+        <v/>
+      </c>
+      <c r="N37">
+        <f>M37*L37</f>
+        <v/>
+      </c>
+      <c r="P37" s="2">
         <f>LOOKUP(A37,Cambi!$A$2:$A$255,Cambi!$A$2:$A$255)</f>
-        <v/>
-      </c>
-      <c r="H37">
-        <f>IF(C37="","",C37/F37)</f>
-        <v/>
-      </c>
-      <c r="I37">
-        <f>IF(D37="","",D37/F37)</f>
-        <v/>
-      </c>
-      <c r="J37">
-        <f>J36+N(H37)-N(I37)</f>
-        <v/>
-      </c>
-      <c r="K37">
-        <f>A38-A37</f>
-        <v/>
-      </c>
-      <c r="L37">
-        <f>K37*J37</f>
         <v/>
       </c>
     </row>
@@ -1992,35 +2153,39 @@
         <v>1000</v>
       </c>
       <c r="E38">
-        <f>E37+N(C38)-N(D38)</f>
-        <v/>
-      </c>
-      <c r="F38">
+        <f>E37+C38-D38</f>
+        <v/>
+      </c>
+      <c r="F38" s="3">
+        <f>DAYS(A39,A38)</f>
+        <v/>
+      </c>
+      <c r="G38">
+        <f>F38*E38</f>
+        <v/>
+      </c>
+      <c r="I38">
         <f>LOOKUP(A38,Cambi!$A$2:$A$255,Cambi!$B$2:$B$255)</f>
         <v/>
       </c>
-      <c r="G38" s="2">
+      <c r="J38">
+        <f>C38/I38</f>
+        <v/>
+      </c>
+      <c r="L38">
+        <f>L37+J38-K38</f>
+        <v/>
+      </c>
+      <c r="M38" s="3">
+        <f>F38</f>
+        <v/>
+      </c>
+      <c r="N38">
+        <f>M38*L38</f>
+        <v/>
+      </c>
+      <c r="P38" s="2">
         <f>LOOKUP(A38,Cambi!$A$2:$A$255,Cambi!$A$2:$A$255)</f>
-        <v/>
-      </c>
-      <c r="H38">
-        <f>IF(C38="","",C38/F38)</f>
-        <v/>
-      </c>
-      <c r="I38">
-        <f>IF(D38="","",D38/F38)</f>
-        <v/>
-      </c>
-      <c r="J38">
-        <f>J37+N(H38)-N(I38)</f>
-        <v/>
-      </c>
-      <c r="K38">
-        <f>A39-A38</f>
-        <v/>
-      </c>
-      <c r="L38">
-        <f>K38*J38</f>
         <v/>
       </c>
     </row>
@@ -2033,35 +2198,39 @@
         <v>600</v>
       </c>
       <c r="E39">
-        <f>E38+N(C39)-N(D39)</f>
-        <v/>
-      </c>
-      <c r="F39">
+        <f>E38+C39-D39</f>
+        <v/>
+      </c>
+      <c r="F39" s="3">
+        <f>DAYS(A40,A39)</f>
+        <v/>
+      </c>
+      <c r="G39">
+        <f>F39*E39</f>
+        <v/>
+      </c>
+      <c r="I39">
         <f>LOOKUP(A39,Cambi!$A$2:$A$255,Cambi!$B$2:$B$255)</f>
         <v/>
       </c>
-      <c r="G39" s="2">
+      <c r="J39">
+        <f>C39/I39</f>
+        <v/>
+      </c>
+      <c r="L39">
+        <f>L38+J39-K39</f>
+        <v/>
+      </c>
+      <c r="M39" s="3">
+        <f>F39</f>
+        <v/>
+      </c>
+      <c r="N39">
+        <f>M39*L39</f>
+        <v/>
+      </c>
+      <c r="P39" s="2">
         <f>LOOKUP(A39,Cambi!$A$2:$A$255,Cambi!$A$2:$A$255)</f>
-        <v/>
-      </c>
-      <c r="H39">
-        <f>IF(C39="","",C39/F39)</f>
-        <v/>
-      </c>
-      <c r="I39">
-        <f>IF(D39="","",D39/F39)</f>
-        <v/>
-      </c>
-      <c r="J39">
-        <f>J38+N(H39)-N(I39)</f>
-        <v/>
-      </c>
-      <c r="K39">
-        <f>A40-A39</f>
-        <v/>
-      </c>
-      <c r="L39">
-        <f>K39*J39</f>
         <v/>
       </c>
     </row>
@@ -2074,35 +2243,39 @@
         <v>1000</v>
       </c>
       <c r="E40">
-        <f>E39+N(C40)-N(D40)</f>
-        <v/>
-      </c>
-      <c r="F40">
+        <f>E39+C40-D40</f>
+        <v/>
+      </c>
+      <c r="F40" s="3">
+        <f>DAYS(A41,A40)</f>
+        <v/>
+      </c>
+      <c r="G40">
+        <f>F40*E40</f>
+        <v/>
+      </c>
+      <c r="I40">
         <f>LOOKUP(A40,Cambi!$A$2:$A$255,Cambi!$B$2:$B$255)</f>
         <v/>
       </c>
-      <c r="G40" s="2">
+      <c r="J40">
+        <f>C40/I40</f>
+        <v/>
+      </c>
+      <c r="L40">
+        <f>L39+J40-K40</f>
+        <v/>
+      </c>
+      <c r="M40" s="3">
+        <f>F40</f>
+        <v/>
+      </c>
+      <c r="N40">
+        <f>M40*L40</f>
+        <v/>
+      </c>
+      <c r="P40" s="2">
         <f>LOOKUP(A40,Cambi!$A$2:$A$255,Cambi!$A$2:$A$255)</f>
-        <v/>
-      </c>
-      <c r="H40">
-        <f>IF(C40="","",C40/F40)</f>
-        <v/>
-      </c>
-      <c r="I40">
-        <f>IF(D40="","",D40/F40)</f>
-        <v/>
-      </c>
-      <c r="J40">
-        <f>J39+N(H40)-N(I40)</f>
-        <v/>
-      </c>
-      <c r="K40">
-        <f>A41-A40</f>
-        <v/>
-      </c>
-      <c r="L40">
-        <f>K40*J40</f>
         <v/>
       </c>
     </row>
@@ -2115,35 +2288,39 @@
         <v>2000</v>
       </c>
       <c r="E41">
-        <f>E40+N(C41)-N(D41)</f>
-        <v/>
-      </c>
-      <c r="F41">
+        <f>E40+C41-D41</f>
+        <v/>
+      </c>
+      <c r="F41" s="3">
+        <f>DAYS(A42,A41)</f>
+        <v/>
+      </c>
+      <c r="G41">
+        <f>F41*E41</f>
+        <v/>
+      </c>
+      <c r="I41">
         <f>LOOKUP(A41,Cambi!$A$2:$A$255,Cambi!$B$2:$B$255)</f>
         <v/>
       </c>
-      <c r="G41" s="2">
+      <c r="K41">
+        <f>D41/I41</f>
+        <v/>
+      </c>
+      <c r="L41">
+        <f>L40+J41-K41</f>
+        <v/>
+      </c>
+      <c r="M41" s="3">
+        <f>F41</f>
+        <v/>
+      </c>
+      <c r="N41">
+        <f>M41*L41</f>
+        <v/>
+      </c>
+      <c r="P41" s="2">
         <f>LOOKUP(A41,Cambi!$A$2:$A$255,Cambi!$A$2:$A$255)</f>
-        <v/>
-      </c>
-      <c r="H41">
-        <f>IF(C41="","",C41/F41)</f>
-        <v/>
-      </c>
-      <c r="I41">
-        <f>IF(D41="","",D41/F41)</f>
-        <v/>
-      </c>
-      <c r="J41">
-        <f>J40+N(H41)-N(I41)</f>
-        <v/>
-      </c>
-      <c r="K41">
-        <f>A42-A41</f>
-        <v/>
-      </c>
-      <c r="L41">
-        <f>K41*J41</f>
         <v/>
       </c>
     </row>
@@ -2156,35 +2333,39 @@
         <v>600</v>
       </c>
       <c r="E42">
-        <f>E41+N(C42)-N(D42)</f>
-        <v/>
-      </c>
-      <c r="F42">
+        <f>E41+C42-D42</f>
+        <v/>
+      </c>
+      <c r="F42" s="3">
+        <f>DAYS(A43,A42)</f>
+        <v/>
+      </c>
+      <c r="G42">
+        <f>F42*E42</f>
+        <v/>
+      </c>
+      <c r="I42">
         <f>LOOKUP(A42,Cambi!$A$2:$A$255,Cambi!$B$2:$B$255)</f>
         <v/>
       </c>
-      <c r="G42" s="2">
+      <c r="J42">
+        <f>C42/I42</f>
+        <v/>
+      </c>
+      <c r="L42">
+        <f>L41+J42-K42</f>
+        <v/>
+      </c>
+      <c r="M42" s="3">
+        <f>F42</f>
+        <v/>
+      </c>
+      <c r="N42">
+        <f>M42*L42</f>
+        <v/>
+      </c>
+      <c r="P42" s="2">
         <f>LOOKUP(A42,Cambi!$A$2:$A$255,Cambi!$A$2:$A$255)</f>
-        <v/>
-      </c>
-      <c r="H42">
-        <f>IF(C42="","",C42/F42)</f>
-        <v/>
-      </c>
-      <c r="I42">
-        <f>IF(D42="","",D42/F42)</f>
-        <v/>
-      </c>
-      <c r="J42">
-        <f>J41+N(H42)-N(I42)</f>
-        <v/>
-      </c>
-      <c r="K42">
-        <f>A43-A42</f>
-        <v/>
-      </c>
-      <c r="L42">
-        <f>K42*J42</f>
         <v/>
       </c>
     </row>
@@ -2197,35 +2378,39 @@
         <v>1768.3</v>
       </c>
       <c r="E43">
-        <f>E42+N(C43)-N(D43)</f>
-        <v/>
-      </c>
-      <c r="F43">
+        <f>E42+C43-D43</f>
+        <v/>
+      </c>
+      <c r="F43" s="3">
+        <f>DAYS(A44,A43)</f>
+        <v/>
+      </c>
+      <c r="G43">
+        <f>F43*E43</f>
+        <v/>
+      </c>
+      <c r="I43">
         <f>LOOKUP(A43,Cambi!$A$2:$A$255,Cambi!$B$2:$B$255)</f>
         <v/>
       </c>
-      <c r="G43" s="2">
+      <c r="K43">
+        <f>D43/I43</f>
+        <v/>
+      </c>
+      <c r="L43">
+        <f>L42+J43-K43</f>
+        <v/>
+      </c>
+      <c r="M43" s="3">
+        <f>F43</f>
+        <v/>
+      </c>
+      <c r="N43">
+        <f>M43*L43</f>
+        <v/>
+      </c>
+      <c r="P43" s="2">
         <f>LOOKUP(A43,Cambi!$A$2:$A$255,Cambi!$A$2:$A$255)</f>
-        <v/>
-      </c>
-      <c r="H43">
-        <f>IF(C43="","",C43/F43)</f>
-        <v/>
-      </c>
-      <c r="I43">
-        <f>IF(D43="","",D43/F43)</f>
-        <v/>
-      </c>
-      <c r="J43">
-        <f>J42+N(H43)-N(I43)</f>
-        <v/>
-      </c>
-      <c r="K43">
-        <f>A44-A43</f>
-        <v/>
-      </c>
-      <c r="L43">
-        <f>K43*J43</f>
         <v/>
       </c>
     </row>
@@ -2238,35 +2423,39 @@
         <v>1000</v>
       </c>
       <c r="E44">
-        <f>E43+N(C44)-N(D44)</f>
-        <v/>
-      </c>
-      <c r="F44">
+        <f>E43+C44-D44</f>
+        <v/>
+      </c>
+      <c r="F44" s="3">
+        <f>DAYS(A45,A44)</f>
+        <v/>
+      </c>
+      <c r="G44">
+        <f>F44*E44</f>
+        <v/>
+      </c>
+      <c r="I44">
         <f>LOOKUP(A44,Cambi!$A$2:$A$255,Cambi!$B$2:$B$255)</f>
         <v/>
       </c>
-      <c r="G44" s="2">
+      <c r="J44">
+        <f>C44/I44</f>
+        <v/>
+      </c>
+      <c r="L44">
+        <f>L43+J44-K44</f>
+        <v/>
+      </c>
+      <c r="M44" s="3">
+        <f>F44</f>
+        <v/>
+      </c>
+      <c r="N44">
+        <f>M44*L44</f>
+        <v/>
+      </c>
+      <c r="P44" s="2">
         <f>LOOKUP(A44,Cambi!$A$2:$A$255,Cambi!$A$2:$A$255)</f>
-        <v/>
-      </c>
-      <c r="H44">
-        <f>IF(C44="","",C44/F44)</f>
-        <v/>
-      </c>
-      <c r="I44">
-        <f>IF(D44="","",D44/F44)</f>
-        <v/>
-      </c>
-      <c r="J44">
-        <f>J43+N(H44)-N(I44)</f>
-        <v/>
-      </c>
-      <c r="K44">
-        <f>A45-A44</f>
-        <v/>
-      </c>
-      <c r="L44">
-        <f>K44*J44</f>
         <v/>
       </c>
     </row>
@@ -2279,35 +2468,38 @@
         <v>600</v>
       </c>
       <c r="E45">
-        <f>E44+N(C45)-N(D45)</f>
-        <v/>
-      </c>
-      <c r="F45">
+        <f>E44+C45-D45</f>
+        <v/>
+      </c>
+      <c r="F45" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="G45">
+        <f>F45*E45</f>
+        <v/>
+      </c>
+      <c r="I45">
         <f>LOOKUP(A45,Cambi!$A$2:$A$255,Cambi!$B$2:$B$255)</f>
         <v/>
       </c>
-      <c r="G45" s="2">
+      <c r="J45">
+        <f>C45/I45</f>
+        <v/>
+      </c>
+      <c r="L45">
+        <f>L44+J45-K45</f>
+        <v/>
+      </c>
+      <c r="M45" s="3">
+        <f>F45</f>
+        <v/>
+      </c>
+      <c r="N45">
+        <f>M45*L45</f>
+        <v/>
+      </c>
+      <c r="P45" s="2">
         <f>LOOKUP(A45,Cambi!$A$2:$A$255,Cambi!$A$2:$A$255)</f>
-        <v/>
-      </c>
-      <c r="H45">
-        <f>IF(C45="","",C45/F45)</f>
-        <v/>
-      </c>
-      <c r="I45">
-        <f>IF(D45="","",D45/F45)</f>
-        <v/>
-      </c>
-      <c r="J45">
-        <f>J44+N(H45)-N(I45)</f>
-        <v/>
-      </c>
-      <c r="K45">
-        <f>DATE(YEAR(A45),12,31)-A45</f>
-        <v/>
-      </c>
-      <c r="L45">
-        <f>K45*J45</f>
         <v/>
       </c>
     </row>
@@ -2317,8 +2509,8 @@
           <t>giacenza media (EUR)</t>
         </is>
       </c>
-      <c r="J47">
-        <f>SUM(L2:L45)/SUM(K2:K45)</f>
+      <c r="N47">
+        <f>SUM(N2:N45)/SUM(M2:M45)</f>
         <v/>
       </c>
     </row>

</xml_diff>